<commit_message>
Add equivalent-elevation and elevation-delta outputs to great lakes TWL batch tooling
</commit_message>
<xml_diff>
--- a/examples/great_lakes/longtailpoint/batch_twl-nointerpolation.xlsx
+++ b/examples/great_lakes/longtailpoint/batch_twl-nointerpolation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="resources"/>
@@ -219,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -239,7 +239,7 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -249,9 +249,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
@@ -589,14 +586,14 @@
     <col min="1" max="1" style="3" width="14.862142857142858" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="3" width="17.433571428571426" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -662,7 +659,7 @@
       <c r="I2" s="10">
         <v>178.7747637915269</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="10">
         <v>178.47</v>
       </c>
       <c r="K2" s="10">
@@ -697,7 +694,7 @@
       <c r="I3" s="10">
         <v>178.1651935385553</v>
       </c>
-      <c r="J3" s="11">
+      <c r="J3" s="10">
         <v>178.47</v>
       </c>
       <c r="K3" s="10">
@@ -732,7 +729,7 @@
       <c r="I4" s="10">
         <v>178.0128009753124</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="10">
         <v>178.47</v>
       </c>
       <c r="K4" s="10">
@@ -767,7 +764,7 @@
       <c r="I5" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="10">
         <v>178.47</v>
       </c>
       <c r="K5" s="10">
@@ -775,34 +772,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="13">
+      <c r="C6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="12">
         <v>1968</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G6" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" s="15">
+      <c r="G6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="14">
         <v>178.622371228284</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="10">
         <v>178.47</v>
       </c>
       <c r="K6" s="10">
@@ -810,34 +807,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="13">
+      <c r="C7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="12">
         <v>1968</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G7" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" s="15">
+      <c r="G7" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="14">
         <v>178.0128009753124</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="10">
         <v>178.47</v>
       </c>
       <c r="K7" s="10">
@@ -845,34 +842,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="13">
+      <c r="C8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="12">
         <v>1968</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G8" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I8" s="15">
+      <c r="G8" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="14">
         <v>177.8604084120695</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="10">
         <v>178.47</v>
       </c>
       <c r="K8" s="10">
@@ -880,34 +877,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="13">
+      <c r="C9" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="12">
         <v>1968</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G9" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I9" s="15">
+      <c r="G9" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="10">
         <v>178.47</v>
       </c>
       <c r="K9" s="10">
@@ -942,7 +939,7 @@
       <c r="I10" s="10">
         <v>178.4699786650411</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="10">
         <v>178.47</v>
       </c>
       <c r="K10" s="10">
@@ -977,7 +974,7 @@
       <c r="I11" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="10">
         <v>178.47</v>
       </c>
       <c r="K11" s="10">
@@ -1012,7 +1009,7 @@
       <c r="I12" s="10">
         <v>177.7080158488266</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="10">
         <v>178.47</v>
       </c>
       <c r="K12" s="10">
@@ -1047,7 +1044,7 @@
       <c r="I13" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="10">
         <v>178.47</v>
       </c>
       <c r="K13" s="10">
@@ -1055,34 +1052,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="13">
+      <c r="C14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="12">
         <v>1968</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G14" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I14" s="15">
+      <c r="G14" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="14">
         <v>178.3175861017982</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="10">
         <v>178.47</v>
       </c>
       <c r="K14" s="10">
@@ -1090,34 +1087,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="13">
+      <c r="C15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="12">
         <v>1968</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G15" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" s="15">
+      <c r="G15" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="10">
         <v>178.47</v>
       </c>
       <c r="K15" s="10">
@@ -1125,34 +1122,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="13">
+      <c r="C16" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="12">
         <v>1968</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F16" s="14">
+      <c r="F16" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G16" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I16" s="15">
+      <c r="G16" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="14">
         <v>177.5556232855836</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="10">
         <v>178.47</v>
       </c>
       <c r="K16" s="10">
@@ -1160,34 +1157,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="13">
+      <c r="C17" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="12">
         <v>1968</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G17" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" s="15">
+      <c r="G17" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="10">
         <v>178.47</v>
       </c>
       <c r="K17" s="10">
@@ -1222,14 +1219,14 @@
       <c r="I18" s="10">
         <v>178.1651935385553</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="10">
         <v>178.47</v>
       </c>
       <c r="K18" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="2" t="s">
         <v>35</v>
       </c>
@@ -1257,14 +1254,14 @@
       <c r="I19" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="10">
         <v>178.47</v>
       </c>
       <c r="K19" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1292,14 +1289,14 @@
       <c r="I20" s="10">
         <v>177.4032307223407</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20" s="10">
         <v>178.47</v>
       </c>
       <c r="K20" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="2" t="s">
         <v>35</v>
       </c>
@@ -1327,154 +1324,154 @@
       <c r="I21" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21" s="10">
         <v>178.47</v>
       </c>
       <c r="K21" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+      <c r="A22" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="13">
+      <c r="C22" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="12">
         <v>1968</v>
       </c>
-      <c r="E22" s="14">
+      <c r="E22" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G22" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="15">
+      <c r="G22" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I22" s="14">
         <v>178.0128009753124</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22" s="10">
         <v>178.47</v>
       </c>
       <c r="K22" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
+      <c r="A23" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="13">
+      <c r="C23" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="12">
         <v>1968</v>
       </c>
-      <c r="E23" s="14">
+      <c r="E23" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F23" s="14">
+      <c r="F23" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G23" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I23" s="15">
+      <c r="G23" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I23" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23" s="10">
         <v>178.47</v>
       </c>
       <c r="K23" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
+      <c r="A24" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="13">
+      <c r="C24" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="12">
         <v>1968</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F24" s="14">
+      <c r="F24" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G24" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I24" s="15">
+      <c r="G24" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="14">
         <v>177.2508381590978</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24" s="10">
         <v>178.47</v>
       </c>
       <c r="K24" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
+      <c r="A25" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C25" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="13">
+      <c r="C25" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="12">
         <v>1968</v>
       </c>
-      <c r="E25" s="14">
+      <c r="E25" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F25" s="14">
+      <c r="F25" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G25" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I25" s="15">
+      <c r="G25" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I25" s="14">
         <v>177.0984455958549</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25" s="10">
         <v>178.47</v>
       </c>
       <c r="K25" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="2" t="s">
         <v>37</v>
       </c>
@@ -1502,14 +1499,14 @@
       <c r="I26" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26" s="10">
         <v>178.47</v>
       </c>
       <c r="K26" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="2" t="s">
         <v>37</v>
       </c>
@@ -1537,14 +1534,14 @@
       <c r="I27" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27" s="10">
         <v>178.47</v>
       </c>
       <c r="K27" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="2" t="s">
         <v>37</v>
       </c>
@@ -1572,14 +1569,14 @@
       <c r="I28" s="10">
         <v>177.0984455958549</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28" s="10">
         <v>178.47</v>
       </c>
       <c r="K28" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="2" t="s">
         <v>37</v>
       </c>
@@ -1607,154 +1604,154 @@
       <c r="I29" s="10">
         <v>176.946053032612</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29" s="10">
         <v>178.47</v>
       </c>
       <c r="K29" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
+      <c r="A30" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="13">
+      <c r="C30" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="12">
         <v>1968</v>
       </c>
-      <c r="E30" s="14">
+      <c r="E30" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F30" s="14">
+      <c r="F30" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G30" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I30" s="15">
+      <c r="G30" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I30" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="10">
         <v>178.47</v>
       </c>
       <c r="K30" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
+      <c r="A31" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D31" s="13">
+      <c r="C31" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="12">
         <v>1968</v>
       </c>
-      <c r="E31" s="14">
+      <c r="E31" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F31" s="14">
+      <c r="F31" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G31" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H31" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I31" s="15">
+      <c r="G31" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I31" s="14">
         <v>177.0984455958549</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="10">
         <v>178.47</v>
       </c>
       <c r="K31" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
+      <c r="A32" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="13">
+      <c r="C32" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="12">
         <v>1968</v>
       </c>
-      <c r="E32" s="14">
+      <c r="E32" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F32" s="14">
+      <c r="F32" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G32" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H32" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I32" s="15">
+      <c r="G32" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I32" s="14">
         <v>176.946053032612</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="10">
         <v>178.47</v>
       </c>
       <c r="K32" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
+      <c r="A33" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D33" s="13">
+      <c r="C33" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="12">
         <v>1968</v>
       </c>
-      <c r="E33" s="14">
+      <c r="E33" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F33" s="14">
+      <c r="F33" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G33" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I33" s="15">
+      <c r="G33" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I33" s="14">
         <v>176.7936604693691</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="10">
         <v>178.47</v>
       </c>
       <c r="K33" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
       <c r="A34" s="2" t="s">
         <v>39</v>
       </c>
@@ -1782,14 +1779,14 @@
       <c r="I34" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34" s="10">
         <v>178.47</v>
       </c>
       <c r="K34" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5">
       <c r="A35" s="2" t="s">
         <v>39</v>
       </c>
@@ -1817,14 +1814,14 @@
       <c r="I35" s="10">
         <v>176.946053032612</v>
       </c>
-      <c r="J35" s="11">
+      <c r="J35" s="10">
         <v>178.47</v>
       </c>
       <c r="K35" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
       <c r="A36" s="2" t="s">
         <v>39</v>
       </c>
@@ -1852,14 +1849,14 @@
       <c r="I36" s="10">
         <v>176.7936604693691</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J36" s="10">
         <v>178.47</v>
       </c>
       <c r="K36" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
       <c r="A37" s="2" t="s">
         <v>39</v>
       </c>
@@ -1887,77 +1884,77 @@
       <c r="I37" s="10">
         <v>176.6412679061262</v>
       </c>
-      <c r="J37" s="11">
+      <c r="J37" s="10">
         <v>178.47</v>
       </c>
       <c r="K37" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
+      <c r="A38" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C38" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D38" s="13">
+      <c r="C38" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38" s="12">
         <v>1968</v>
       </c>
-      <c r="E38" s="14">
+      <c r="E38" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F38" s="14">
+      <c r="F38" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G38" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I38" s="15">
+      <c r="G38" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H38" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I38" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J38" s="11">
+      <c r="J38" s="10">
         <v>178.47</v>
       </c>
       <c r="K38" s="10">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="12" t="s">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="19.5">
+      <c r="A39" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C39" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D39" s="13">
+      <c r="C39" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39" s="12">
         <v>1968</v>
       </c>
-      <c r="E39" s="14">
+      <c r="E39" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F39" s="14">
+      <c r="F39" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G39" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I39" s="15">
+      <c r="G39" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H39" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I39" s="14">
         <v>176.7936604693691</v>
       </c>
-      <c r="J39" s="11">
+      <c r="J39" s="10">
         <v>178.47</v>
       </c>
       <c r="K39" s="10">
@@ -1965,34 +1962,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="13">
+      <c r="C40" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="12">
         <v>1968</v>
       </c>
-      <c r="E40" s="14">
+      <c r="E40" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F40" s="14">
+      <c r="F40" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G40" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H40" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I40" s="15">
+      <c r="G40" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H40" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I40" s="14">
         <v>176.6412679061262</v>
       </c>
-      <c r="J40" s="11">
+      <c r="J40" s="10">
         <v>178.47</v>
       </c>
       <c r="K40" s="10">
@@ -2000,34 +1997,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D41" s="13">
+      <c r="C41" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D41" s="12">
         <v>1968</v>
       </c>
-      <c r="E41" s="14">
+      <c r="E41" s="13">
         <v>44.30264</v>
       </c>
-      <c r="F41" s="14">
+      <c r="F41" s="13">
         <v>-76.0876408</v>
       </c>
-      <c r="G41" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H41" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I41" s="15">
+      <c r="G41" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I41" s="14">
         <v>176.4888753428832</v>
       </c>
-      <c r="J41" s="11">
+      <c r="J41" s="10">
         <v>178.47</v>
       </c>
       <c r="K41" s="10">
@@ -2062,7 +2059,7 @@
       <c r="I42" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42" s="10">
         <v>178.47</v>
       </c>
       <c r="K42" s="10">
@@ -2097,7 +2094,7 @@
       <c r="I43" s="10">
         <v>176.6412679061262</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43" s="10">
         <v>178.47</v>
       </c>
       <c r="K43" s="10">
@@ -2132,7 +2129,7 @@
       <c r="I44" s="10">
         <v>176.4888753428832</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44" s="10">
         <v>178.47</v>
       </c>
       <c r="K44" s="10">
@@ -2167,7 +2164,7 @@
       <c r="I45" s="10">
         <v>176.3364827796403</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45" s="10">
         <v>178.47</v>
       </c>
       <c r="K45" s="10">
@@ -2202,7 +2199,7 @@
       <c r="I46" s="10">
         <v>178.7747637915269</v>
       </c>
-      <c r="J46" s="11">
+      <c r="J46" s="10">
         <v>178.47</v>
       </c>
       <c r="K46" s="10">
@@ -2237,7 +2234,7 @@
       <c r="I47" s="10">
         <v>178.1651935385553</v>
       </c>
-      <c r="J47" s="11">
+      <c r="J47" s="10">
         <v>178.47</v>
       </c>
       <c r="K47" s="10">
@@ -2272,7 +2269,7 @@
       <c r="I48" s="10">
         <v>178.0128009753124</v>
       </c>
-      <c r="J48" s="11">
+      <c r="J48" s="10">
         <v>178.47</v>
       </c>
       <c r="K48" s="10">
@@ -2307,7 +2304,7 @@
       <c r="I49" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J49" s="11">
+      <c r="J49" s="10">
         <v>178.47</v>
       </c>
       <c r="K49" s="10">
@@ -2315,34 +2312,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="12" t="s">
+      <c r="A50" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C50" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D50" s="13">
+      <c r="C50" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D50" s="12">
         <v>4997</v>
       </c>
-      <c r="E50" s="14">
+      <c r="E50" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F50" s="14">
+      <c r="F50" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G50" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H50" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I50" s="15">
+      <c r="G50" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H50" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I50" s="14">
         <v>178.622371228284</v>
       </c>
-      <c r="J50" s="11">
+      <c r="J50" s="10">
         <v>178.47</v>
       </c>
       <c r="K50" s="10">
@@ -2350,34 +2347,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C51" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D51" s="13">
+      <c r="C51" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" s="12">
         <v>4997</v>
       </c>
-      <c r="E51" s="14">
+      <c r="E51" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F51" s="14">
+      <c r="F51" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G51" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H51" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I51" s="15">
+      <c r="G51" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H51" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I51" s="14">
         <v>178.0128009753124</v>
       </c>
-      <c r="J51" s="11">
+      <c r="J51" s="10">
         <v>178.47</v>
       </c>
       <c r="K51" s="10">
@@ -2385,34 +2382,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="12" t="s">
+      <c r="A52" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B52" s="12" t="s">
+      <c r="B52" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C52" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D52" s="13">
+      <c r="C52" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="12">
         <v>4997</v>
       </c>
-      <c r="E52" s="14">
+      <c r="E52" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F52" s="14">
+      <c r="F52" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G52" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H52" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I52" s="15">
+      <c r="G52" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H52" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I52" s="14">
         <v>177.8604084120695</v>
       </c>
-      <c r="J52" s="11">
+      <c r="J52" s="10">
         <v>178.47</v>
       </c>
       <c r="K52" s="10">
@@ -2420,34 +2417,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="12" t="s">
+      <c r="A53" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B53" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D53" s="13">
+      <c r="C53" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D53" s="12">
         <v>4997</v>
       </c>
-      <c r="E53" s="14">
+      <c r="E53" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F53" s="14">
+      <c r="F53" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G53" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H53" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I53" s="15">
+      <c r="G53" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H53" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I53" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J53" s="11">
+      <c r="J53" s="10">
         <v>178.47</v>
       </c>
       <c r="K53" s="10">
@@ -2482,7 +2479,7 @@
       <c r="I54" s="10">
         <v>178.4699786650411</v>
       </c>
-      <c r="J54" s="11">
+      <c r="J54" s="10">
         <v>178.47</v>
       </c>
       <c r="K54" s="10">
@@ -2517,7 +2514,7 @@
       <c r="I55" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J55" s="11">
+      <c r="J55" s="10">
         <v>178.47</v>
       </c>
       <c r="K55" s="10">
@@ -2552,7 +2549,7 @@
       <c r="I56" s="10">
         <v>177.7080158488266</v>
       </c>
-      <c r="J56" s="11">
+      <c r="J56" s="10">
         <v>178.47</v>
       </c>
       <c r="K56" s="10">
@@ -2587,7 +2584,7 @@
       <c r="I57" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J57" s="11">
+      <c r="J57" s="10">
         <v>178.47</v>
       </c>
       <c r="K57" s="10">
@@ -2595,34 +2592,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D58" s="13">
+      <c r="C58" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D58" s="12">
         <v>4997</v>
       </c>
-      <c r="E58" s="14">
+      <c r="E58" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F58" s="14">
+      <c r="F58" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G58" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H58" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I58" s="15">
+      <c r="G58" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H58" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I58" s="14">
         <v>178.3175861017982</v>
       </c>
-      <c r="J58" s="11">
+      <c r="J58" s="10">
         <v>178.47</v>
       </c>
       <c r="K58" s="10">
@@ -2630,34 +2627,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C59" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D59" s="13">
+      <c r="C59" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D59" s="12">
         <v>4997</v>
       </c>
-      <c r="E59" s="14">
+      <c r="E59" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F59" s="14">
+      <c r="F59" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G59" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H59" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I59" s="15">
+      <c r="G59" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H59" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I59" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J59" s="11">
+      <c r="J59" s="10">
         <v>178.47</v>
       </c>
       <c r="K59" s="10">
@@ -2665,34 +2662,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="12" t="s">
+      <c r="A60" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B60" s="12" t="s">
+      <c r="B60" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C60" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D60" s="13">
+      <c r="C60" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D60" s="12">
         <v>4997</v>
       </c>
-      <c r="E60" s="14">
+      <c r="E60" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F60" s="14">
+      <c r="F60" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G60" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H60" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I60" s="15">
+      <c r="G60" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H60" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I60" s="14">
         <v>177.5556232855836</v>
       </c>
-      <c r="J60" s="11">
+      <c r="J60" s="10">
         <v>178.47</v>
       </c>
       <c r="K60" s="10">
@@ -2700,34 +2697,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D61" s="13">
+      <c r="C61" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D61" s="12">
         <v>4997</v>
       </c>
-      <c r="E61" s="14">
+      <c r="E61" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F61" s="14">
+      <c r="F61" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G61" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H61" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I61" s="15">
+      <c r="G61" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H61" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I61" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J61" s="11">
+      <c r="J61" s="10">
         <v>178.47</v>
       </c>
       <c r="K61" s="10">
@@ -2762,7 +2759,7 @@
       <c r="I62" s="10">
         <v>178.1651935385553</v>
       </c>
-      <c r="J62" s="11">
+      <c r="J62" s="10">
         <v>178.47</v>
       </c>
       <c r="K62" s="10">
@@ -2797,7 +2794,7 @@
       <c r="I63" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J63" s="11">
+      <c r="J63" s="10">
         <v>178.47</v>
       </c>
       <c r="K63" s="10">
@@ -2832,7 +2829,7 @@
       <c r="I64" s="10">
         <v>177.4032307223407</v>
       </c>
-      <c r="J64" s="11">
+      <c r="J64" s="10">
         <v>178.47</v>
       </c>
       <c r="K64" s="10">
@@ -2867,7 +2864,7 @@
       <c r="I65" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J65" s="11">
+      <c r="J65" s="10">
         <v>178.47</v>
       </c>
       <c r="K65" s="10">
@@ -2875,34 +2872,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B66" s="12" t="s">
+      <c r="B66" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C66" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D66" s="13">
+      <c r="C66" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D66" s="12">
         <v>4997</v>
       </c>
-      <c r="E66" s="14">
+      <c r="E66" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F66" s="14">
+      <c r="F66" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G66" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H66" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I66" s="15">
+      <c r="G66" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H66" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I66" s="14">
         <v>178.0128009753124</v>
       </c>
-      <c r="J66" s="11">
+      <c r="J66" s="10">
         <v>178.47</v>
       </c>
       <c r="K66" s="10">
@@ -2910,34 +2907,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D67" s="13">
+      <c r="C67" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D67" s="12">
         <v>4997</v>
       </c>
-      <c r="E67" s="14">
+      <c r="E67" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F67" s="14">
+      <c r="F67" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G67" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H67" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I67" s="15">
+      <c r="G67" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H67" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I67" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J67" s="11">
+      <c r="J67" s="10">
         <v>178.47</v>
       </c>
       <c r="K67" s="10">
@@ -2945,34 +2942,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="12" t="s">
+      <c r="A68" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B68" s="12" t="s">
+      <c r="B68" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C68" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D68" s="13">
+      <c r="C68" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D68" s="12">
         <v>4997</v>
       </c>
-      <c r="E68" s="14">
+      <c r="E68" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F68" s="14">
+      <c r="F68" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G68" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H68" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I68" s="15">
+      <c r="G68" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H68" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I68" s="14">
         <v>177.2508381590978</v>
       </c>
-      <c r="J68" s="11">
+      <c r="J68" s="10">
         <v>178.47</v>
       </c>
       <c r="K68" s="10">
@@ -2980,34 +2977,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="12" t="s">
+      <c r="A69" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C69" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D69" s="13">
+      <c r="C69" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D69" s="12">
         <v>4997</v>
       </c>
-      <c r="E69" s="14">
+      <c r="E69" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F69" s="14">
+      <c r="F69" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G69" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H69" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I69" s="15">
+      <c r="G69" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H69" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I69" s="14">
         <v>177.0984455958549</v>
       </c>
-      <c r="J69" s="11">
+      <c r="J69" s="10">
         <v>178.47</v>
       </c>
       <c r="K69" s="10">
@@ -3042,7 +3039,7 @@
       <c r="I70" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J70" s="11">
+      <c r="J70" s="10">
         <v>178.47</v>
       </c>
       <c r="K70" s="10">
@@ -3077,7 +3074,7 @@
       <c r="I71" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J71" s="11">
+      <c r="J71" s="10">
         <v>178.47</v>
       </c>
       <c r="K71" s="10">
@@ -3112,7 +3109,7 @@
       <c r="I72" s="10">
         <v>177.0984455958549</v>
       </c>
-      <c r="J72" s="11">
+      <c r="J72" s="10">
         <v>178.47</v>
       </c>
       <c r="K72" s="10">
@@ -3147,7 +3144,7 @@
       <c r="I73" s="10">
         <v>176.946053032612</v>
       </c>
-      <c r="J73" s="11">
+      <c r="J73" s="10">
         <v>178.47</v>
       </c>
       <c r="K73" s="10">
@@ -3155,34 +3152,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="12" t="s">
+      <c r="A74" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B74" s="12" t="s">
+      <c r="B74" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C74" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D74" s="13">
+      <c r="C74" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D74" s="12">
         <v>4997</v>
       </c>
-      <c r="E74" s="14">
+      <c r="E74" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F74" s="14">
+      <c r="F74" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G74" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H74" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I74" s="15">
+      <c r="G74" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H74" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I74" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J74" s="11">
+      <c r="J74" s="10">
         <v>178.47</v>
       </c>
       <c r="K74" s="10">
@@ -3190,34 +3187,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="12" t="s">
+      <c r="A75" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="12" t="s">
+      <c r="B75" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C75" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D75" s="13">
+      <c r="C75" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D75" s="12">
         <v>4997</v>
       </c>
-      <c r="E75" s="14">
+      <c r="E75" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F75" s="14">
+      <c r="F75" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G75" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H75" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I75" s="15">
+      <c r="G75" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H75" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I75" s="14">
         <v>177.0984455958549</v>
       </c>
-      <c r="J75" s="11">
+      <c r="J75" s="10">
         <v>178.47</v>
       </c>
       <c r="K75" s="10">
@@ -3225,34 +3222,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="12" t="s">
+      <c r="A76" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C76" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D76" s="13">
+      <c r="C76" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D76" s="12">
         <v>4997</v>
       </c>
-      <c r="E76" s="14">
+      <c r="E76" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F76" s="14">
+      <c r="F76" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G76" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H76" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I76" s="15">
+      <c r="G76" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H76" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I76" s="14">
         <v>176.946053032612</v>
       </c>
-      <c r="J76" s="11">
+      <c r="J76" s="10">
         <v>178.47</v>
       </c>
       <c r="K76" s="10">
@@ -3260,34 +3257,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="12" t="s">
+      <c r="A77" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C77" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D77" s="13">
+      <c r="C77" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D77" s="12">
         <v>4997</v>
       </c>
-      <c r="E77" s="14">
+      <c r="E77" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F77" s="14">
+      <c r="F77" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G77" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H77" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I77" s="15">
+      <c r="G77" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H77" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I77" s="14">
         <v>176.7936604693691</v>
       </c>
-      <c r="J77" s="11">
+      <c r="J77" s="10">
         <v>178.47</v>
       </c>
       <c r="K77" s="10">
@@ -3322,7 +3319,7 @@
       <c r="I78" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J78" s="11">
+      <c r="J78" s="10">
         <v>178.47</v>
       </c>
       <c r="K78" s="10">
@@ -3357,7 +3354,7 @@
       <c r="I79" s="10">
         <v>176.946053032612</v>
       </c>
-      <c r="J79" s="11">
+      <c r="J79" s="10">
         <v>178.47</v>
       </c>
       <c r="K79" s="10">
@@ -3392,7 +3389,7 @@
       <c r="I80" s="10">
         <v>176.7936604693691</v>
       </c>
-      <c r="J80" s="11">
+      <c r="J80" s="10">
         <v>178.47</v>
       </c>
       <c r="K80" s="10">
@@ -3427,7 +3424,7 @@
       <c r="I81" s="10">
         <v>176.6412679061262</v>
       </c>
-      <c r="J81" s="11">
+      <c r="J81" s="10">
         <v>178.47</v>
       </c>
       <c r="K81" s="10">
@@ -3435,34 +3432,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
-      <c r="A82" s="12" t="s">
+      <c r="A82" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B82" s="12" t="s">
+      <c r="B82" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C82" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D82" s="13">
+      <c r="C82" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D82" s="12">
         <v>4997</v>
       </c>
-      <c r="E82" s="14">
+      <c r="E82" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F82" s="14">
+      <c r="F82" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G82" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H82" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I82" s="15">
+      <c r="G82" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H82" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I82" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J82" s="11">
+      <c r="J82" s="10">
         <v>178.47</v>
       </c>
       <c r="K82" s="10">
@@ -3470,34 +3467,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
-      <c r="A83" s="12" t="s">
+      <c r="A83" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C83" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D83" s="13">
+      <c r="C83" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D83" s="12">
         <v>4997</v>
       </c>
-      <c r="E83" s="14">
+      <c r="E83" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F83" s="14">
+      <c r="F83" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G83" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H83" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I83" s="15">
+      <c r="G83" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H83" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I83" s="14">
         <v>176.7936604693691</v>
       </c>
-      <c r="J83" s="11">
+      <c r="J83" s="10">
         <v>178.47</v>
       </c>
       <c r="K83" s="10">
@@ -3505,34 +3502,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
-      <c r="A84" s="12" t="s">
+      <c r="A84" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B84" s="12" t="s">
+      <c r="B84" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C84" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D84" s="13">
+      <c r="C84" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D84" s="12">
         <v>4997</v>
       </c>
-      <c r="E84" s="14">
+      <c r="E84" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F84" s="14">
+      <c r="F84" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G84" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H84" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I84" s="15">
+      <c r="G84" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H84" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I84" s="14">
         <v>176.6412679061262</v>
       </c>
-      <c r="J84" s="11">
+      <c r="J84" s="10">
         <v>178.47</v>
       </c>
       <c r="K84" s="10">
@@ -3540,34 +3537,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
-      <c r="A85" s="12" t="s">
+      <c r="A85" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C85" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D85" s="13">
+      <c r="C85" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D85" s="12">
         <v>4997</v>
       </c>
-      <c r="E85" s="14">
+      <c r="E85" s="13">
         <v>43.9497771</v>
       </c>
-      <c r="F85" s="14">
+      <c r="F85" s="13">
         <v>-76.8559452</v>
       </c>
-      <c r="G85" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H85" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I85" s="15">
+      <c r="G85" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H85" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I85" s="14">
         <v>176.4888753428832</v>
       </c>
-      <c r="J85" s="11">
+      <c r="J85" s="10">
         <v>178.47</v>
       </c>
       <c r="K85" s="10">
@@ -3602,7 +3599,7 @@
       <c r="I86" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J86" s="11">
+      <c r="J86" s="10">
         <v>178.47</v>
       </c>
       <c r="K86" s="10">
@@ -3637,7 +3634,7 @@
       <c r="I87" s="10">
         <v>176.6412679061262</v>
       </c>
-      <c r="J87" s="11">
+      <c r="J87" s="10">
         <v>178.47</v>
       </c>
       <c r="K87" s="10">
@@ -3672,7 +3669,7 @@
       <c r="I88" s="10">
         <v>176.4888753428832</v>
       </c>
-      <c r="J88" s="11">
+      <c r="J88" s="10">
         <v>178.47</v>
       </c>
       <c r="K88" s="10">
@@ -3707,7 +3704,7 @@
       <c r="I89" s="10">
         <v>176.3364827796403</v>
       </c>
-      <c r="J89" s="11">
+      <c r="J89" s="10">
         <v>178.47</v>
       </c>
       <c r="K89" s="10">
@@ -3727,10 +3724,10 @@
       <c r="D90" s="8">
         <v>4999</v>
       </c>
-      <c r="E90" s="16">
+      <c r="E90" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F90" s="16">
+      <c r="F90" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G90" s="1" t="s">
@@ -3742,7 +3739,7 @@
       <c r="I90" s="10">
         <v>178.7747637915269</v>
       </c>
-      <c r="J90" s="11">
+      <c r="J90" s="10">
         <v>178.47</v>
       </c>
       <c r="K90" s="10">
@@ -3762,10 +3759,10 @@
       <c r="D91" s="8">
         <v>4999</v>
       </c>
-      <c r="E91" s="16">
+      <c r="E91" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F91" s="16">
+      <c r="F91" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G91" s="1" t="s">
@@ -3777,7 +3774,7 @@
       <c r="I91" s="10">
         <v>178.1651935385553</v>
       </c>
-      <c r="J91" s="11">
+      <c r="J91" s="10">
         <v>178.47</v>
       </c>
       <c r="K91" s="10">
@@ -3797,10 +3794,10 @@
       <c r="D92" s="8">
         <v>4999</v>
       </c>
-      <c r="E92" s="16">
+      <c r="E92" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F92" s="16">
+      <c r="F92" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G92" s="1" t="s">
@@ -3812,7 +3809,7 @@
       <c r="I92" s="10">
         <v>178.0128009753124</v>
       </c>
-      <c r="J92" s="11">
+      <c r="J92" s="10">
         <v>178.47</v>
       </c>
       <c r="K92" s="10">
@@ -3832,10 +3829,10 @@
       <c r="D93" s="8">
         <v>4999</v>
       </c>
-      <c r="E93" s="16">
+      <c r="E93" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F93" s="16">
+      <c r="F93" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G93" s="1" t="s">
@@ -3847,7 +3844,7 @@
       <c r="I93" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J93" s="11">
+      <c r="J93" s="10">
         <v>178.47</v>
       </c>
       <c r="K93" s="10">
@@ -3855,34 +3852,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
-      <c r="A94" s="12" t="s">
+      <c r="A94" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B94" s="12" t="s">
+      <c r="B94" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C94" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D94" s="13">
+      <c r="C94" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D94" s="12">
         <v>4999</v>
       </c>
-      <c r="E94" s="17">
+      <c r="E94" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F94" s="17">
+      <c r="F94" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G94" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H94" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I94" s="15">
+      <c r="G94" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H94" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I94" s="14">
         <v>178.622371228284</v>
       </c>
-      <c r="J94" s="11">
+      <c r="J94" s="10">
         <v>178.47</v>
       </c>
       <c r="K94" s="10">
@@ -3890,34 +3887,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
-      <c r="A95" s="12" t="s">
+      <c r="A95" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B95" s="12" t="s">
+      <c r="B95" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C95" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D95" s="13">
+      <c r="C95" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D95" s="12">
         <v>4999</v>
       </c>
-      <c r="E95" s="17">
+      <c r="E95" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F95" s="17">
+      <c r="F95" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G95" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H95" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I95" s="15">
+      <c r="G95" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H95" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I95" s="14">
         <v>178.0128009753124</v>
       </c>
-      <c r="J95" s="11">
+      <c r="J95" s="10">
         <v>178.47</v>
       </c>
       <c r="K95" s="10">
@@ -3925,34 +3922,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
-      <c r="A96" s="12" t="s">
+      <c r="A96" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B96" s="12" t="s">
+      <c r="B96" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C96" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D96" s="13">
+      <c r="C96" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D96" s="12">
         <v>4999</v>
       </c>
-      <c r="E96" s="17">
+      <c r="E96" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F96" s="17">
+      <c r="F96" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G96" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H96" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I96" s="15">
+      <c r="G96" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H96" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I96" s="14">
         <v>177.8604084120695</v>
       </c>
-      <c r="J96" s="11">
+      <c r="J96" s="10">
         <v>178.47</v>
       </c>
       <c r="K96" s="10">
@@ -3960,34 +3957,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
-      <c r="A97" s="12" t="s">
+      <c r="A97" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B97" s="12" t="s">
+      <c r="B97" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C97" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D97" s="13">
+      <c r="C97" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D97" s="12">
         <v>4999</v>
       </c>
-      <c r="E97" s="17">
+      <c r="E97" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F97" s="17">
+      <c r="F97" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G97" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H97" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I97" s="15">
+      <c r="G97" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H97" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I97" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J97" s="11">
+      <c r="J97" s="10">
         <v>178.47</v>
       </c>
       <c r="K97" s="10">
@@ -4007,10 +4004,10 @@
       <c r="D98" s="8">
         <v>4999</v>
       </c>
-      <c r="E98" s="16">
+      <c r="E98" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F98" s="16">
+      <c r="F98" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G98" s="2" t="s">
@@ -4022,7 +4019,7 @@
       <c r="I98" s="10">
         <v>178.4699786650411</v>
       </c>
-      <c r="J98" s="11">
+      <c r="J98" s="10">
         <v>178.47</v>
       </c>
       <c r="K98" s="10">
@@ -4042,10 +4039,10 @@
       <c r="D99" s="8">
         <v>4999</v>
       </c>
-      <c r="E99" s="16">
+      <c r="E99" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F99" s="16">
+      <c r="F99" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G99" s="2" t="s">
@@ -4057,7 +4054,7 @@
       <c r="I99" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J99" s="11">
+      <c r="J99" s="10">
         <v>178.47</v>
       </c>
       <c r="K99" s="10">
@@ -4077,10 +4074,10 @@
       <c r="D100" s="8">
         <v>4999</v>
       </c>
-      <c r="E100" s="16">
+      <c r="E100" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F100" s="16">
+      <c r="F100" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G100" s="2" t="s">
@@ -4092,7 +4089,7 @@
       <c r="I100" s="10">
         <v>177.7080158488266</v>
       </c>
-      <c r="J100" s="11">
+      <c r="J100" s="10">
         <v>178.47</v>
       </c>
       <c r="K100" s="10">
@@ -4112,10 +4109,10 @@
       <c r="D101" s="8">
         <v>4999</v>
       </c>
-      <c r="E101" s="16">
+      <c r="E101" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F101" s="16">
+      <c r="F101" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G101" s="2" t="s">
@@ -4127,7 +4124,7 @@
       <c r="I101" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J101" s="11">
+      <c r="J101" s="10">
         <v>178.47</v>
       </c>
       <c r="K101" s="10">
@@ -4135,34 +4132,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
-      <c r="A102" s="12" t="s">
+      <c r="A102" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B102" s="12" t="s">
+      <c r="B102" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C102" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D102" s="13">
+      <c r="C102" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D102" s="12">
         <v>4999</v>
       </c>
-      <c r="E102" s="17">
+      <c r="E102" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F102" s="17">
+      <c r="F102" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G102" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H102" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I102" s="15">
+      <c r="G102" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H102" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I102" s="14">
         <v>178.3175861017982</v>
       </c>
-      <c r="J102" s="11">
+      <c r="J102" s="10">
         <v>178.47</v>
       </c>
       <c r="K102" s="10">
@@ -4170,34 +4167,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
-      <c r="A103" s="12" t="s">
+      <c r="A103" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B103" s="12" t="s">
+      <c r="B103" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C103" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D103" s="13">
+      <c r="C103" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D103" s="12">
         <v>4999</v>
       </c>
-      <c r="E103" s="17">
+      <c r="E103" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F103" s="17">
+      <c r="F103" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G103" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H103" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I103" s="15">
+      <c r="G103" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H103" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I103" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J103" s="11">
+      <c r="J103" s="10">
         <v>178.47</v>
       </c>
       <c r="K103" s="10">
@@ -4205,34 +4202,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
-      <c r="A104" s="12" t="s">
+      <c r="A104" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B104" s="12" t="s">
+      <c r="B104" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C104" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D104" s="13">
+      <c r="C104" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D104" s="12">
         <v>4999</v>
       </c>
-      <c r="E104" s="17">
+      <c r="E104" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F104" s="17">
+      <c r="F104" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G104" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H104" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I104" s="15">
+      <c r="G104" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I104" s="14">
         <v>177.5556232855836</v>
       </c>
-      <c r="J104" s="11">
+      <c r="J104" s="10">
         <v>178.47</v>
       </c>
       <c r="K104" s="10">
@@ -4240,34 +4237,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
-      <c r="A105" s="12" t="s">
+      <c r="A105" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B105" s="12" t="s">
+      <c r="B105" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C105" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D105" s="13">
+      <c r="C105" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D105" s="12">
         <v>4999</v>
       </c>
-      <c r="E105" s="17">
+      <c r="E105" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F105" s="17">
+      <c r="F105" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G105" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H105" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I105" s="15">
+      <c r="G105" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H105" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I105" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J105" s="11">
+      <c r="J105" s="10">
         <v>178.47</v>
       </c>
       <c r="K105" s="10">
@@ -4287,10 +4284,10 @@
       <c r="D106" s="8">
         <v>4999</v>
       </c>
-      <c r="E106" s="16">
+      <c r="E106" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F106" s="16">
+      <c r="F106" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G106" s="2" t="s">
@@ -4302,7 +4299,7 @@
       <c r="I106" s="10">
         <v>178.1651935385553</v>
       </c>
-      <c r="J106" s="11">
+      <c r="J106" s="10">
         <v>178.47</v>
       </c>
       <c r="K106" s="10">
@@ -4322,10 +4319,10 @@
       <c r="D107" s="8">
         <v>4999</v>
       </c>
-      <c r="E107" s="16">
+      <c r="E107" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F107" s="16">
+      <c r="F107" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G107" s="2" t="s">
@@ -4337,7 +4334,7 @@
       <c r="I107" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J107" s="11">
+      <c r="J107" s="10">
         <v>178.47</v>
       </c>
       <c r="K107" s="10">
@@ -4357,10 +4354,10 @@
       <c r="D108" s="8">
         <v>4999</v>
       </c>
-      <c r="E108" s="16">
+      <c r="E108" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F108" s="16">
+      <c r="F108" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G108" s="2" t="s">
@@ -4372,7 +4369,7 @@
       <c r="I108" s="10">
         <v>177.4032307223407</v>
       </c>
-      <c r="J108" s="11">
+      <c r="J108" s="10">
         <v>178.47</v>
       </c>
       <c r="K108" s="10">
@@ -4392,10 +4389,10 @@
       <c r="D109" s="8">
         <v>4999</v>
       </c>
-      <c r="E109" s="16">
+      <c r="E109" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F109" s="16">
+      <c r="F109" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G109" s="2" t="s">
@@ -4407,7 +4404,7 @@
       <c r="I109" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J109" s="11">
+      <c r="J109" s="10">
         <v>178.47</v>
       </c>
       <c r="K109" s="10">
@@ -4415,34 +4412,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
-      <c r="A110" s="12" t="s">
+      <c r="A110" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B110" s="12" t="s">
+      <c r="B110" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C110" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D110" s="13">
+      <c r="C110" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D110" s="12">
         <v>4999</v>
       </c>
-      <c r="E110" s="17">
+      <c r="E110" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F110" s="17">
+      <c r="F110" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G110" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H110" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I110" s="15">
+      <c r="G110" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H110" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I110" s="14">
         <v>178.0128009753124</v>
       </c>
-      <c r="J110" s="11">
+      <c r="J110" s="10">
         <v>178.47</v>
       </c>
       <c r="K110" s="10">
@@ -4450,34 +4447,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
-      <c r="A111" s="12" t="s">
+      <c r="A111" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B111" s="12" t="s">
+      <c r="B111" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C111" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D111" s="13">
+      <c r="C111" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D111" s="12">
         <v>4999</v>
       </c>
-      <c r="E111" s="17">
+      <c r="E111" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F111" s="17">
+      <c r="F111" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G111" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H111" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I111" s="15">
+      <c r="G111" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H111" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I111" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J111" s="11">
+      <c r="J111" s="10">
         <v>178.47</v>
       </c>
       <c r="K111" s="10">
@@ -4485,34 +4482,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
-      <c r="A112" s="12" t="s">
+      <c r="A112" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B112" s="12" t="s">
+      <c r="B112" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C112" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D112" s="13">
+      <c r="C112" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D112" s="12">
         <v>4999</v>
       </c>
-      <c r="E112" s="17">
+      <c r="E112" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F112" s="17">
+      <c r="F112" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G112" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H112" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I112" s="15">
+      <c r="G112" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H112" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I112" s="14">
         <v>177.2508381590978</v>
       </c>
-      <c r="J112" s="11">
+      <c r="J112" s="10">
         <v>178.47</v>
       </c>
       <c r="K112" s="10">
@@ -4520,34 +4517,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
-      <c r="A113" s="12" t="s">
+      <c r="A113" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B113" s="12" t="s">
+      <c r="B113" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C113" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D113" s="13">
+      <c r="C113" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D113" s="12">
         <v>4999</v>
       </c>
-      <c r="E113" s="17">
+      <c r="E113" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F113" s="17">
+      <c r="F113" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G113" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H113" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I113" s="15">
+      <c r="G113" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H113" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I113" s="14">
         <v>177.0984455958549</v>
       </c>
-      <c r="J113" s="11">
+      <c r="J113" s="10">
         <v>178.47</v>
       </c>
       <c r="K113" s="10">
@@ -4567,10 +4564,10 @@
       <c r="D114" s="8">
         <v>4999</v>
       </c>
-      <c r="E114" s="16">
+      <c r="E114" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F114" s="16">
+      <c r="F114" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G114" s="2" t="s">
@@ -4582,7 +4579,7 @@
       <c r="I114" s="10">
         <v>177.8604084120695</v>
       </c>
-      <c r="J114" s="11">
+      <c r="J114" s="10">
         <v>178.47</v>
       </c>
       <c r="K114" s="10">
@@ -4602,10 +4599,10 @@
       <c r="D115" s="8">
         <v>4999</v>
       </c>
-      <c r="E115" s="16">
+      <c r="E115" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F115" s="16">
+      <c r="F115" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G115" s="2" t="s">
@@ -4617,7 +4614,7 @@
       <c r="I115" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J115" s="11">
+      <c r="J115" s="10">
         <v>178.47</v>
       </c>
       <c r="K115" s="10">
@@ -4637,10 +4634,10 @@
       <c r="D116" s="8">
         <v>4999</v>
       </c>
-      <c r="E116" s="16">
+      <c r="E116" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F116" s="16">
+      <c r="F116" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G116" s="2" t="s">
@@ -4652,7 +4649,7 @@
       <c r="I116" s="10">
         <v>177.0984455958549</v>
       </c>
-      <c r="J116" s="11">
+      <c r="J116" s="10">
         <v>178.47</v>
       </c>
       <c r="K116" s="10">
@@ -4672,10 +4669,10 @@
       <c r="D117" s="8">
         <v>4999</v>
       </c>
-      <c r="E117" s="16">
+      <c r="E117" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F117" s="16">
+      <c r="F117" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G117" s="2" t="s">
@@ -4687,7 +4684,7 @@
       <c r="I117" s="10">
         <v>176.946053032612</v>
       </c>
-      <c r="J117" s="11">
+      <c r="J117" s="10">
         <v>178.47</v>
       </c>
       <c r="K117" s="10">
@@ -4695,34 +4692,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
-      <c r="A118" s="12" t="s">
+      <c r="A118" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B118" s="12" t="s">
+      <c r="B118" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C118" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D118" s="13">
+      <c r="C118" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D118" s="12">
         <v>4999</v>
       </c>
-      <c r="E118" s="17">
+      <c r="E118" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F118" s="17">
+      <c r="F118" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G118" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H118" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I118" s="15">
+      <c r="G118" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H118" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I118" s="14">
         <v>177.7080158488266</v>
       </c>
-      <c r="J118" s="11">
+      <c r="J118" s="10">
         <v>178.47</v>
       </c>
       <c r="K118" s="10">
@@ -4730,34 +4727,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
-      <c r="A119" s="12" t="s">
+      <c r="A119" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B119" s="12" t="s">
+      <c r="B119" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C119" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D119" s="13">
+      <c r="C119" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D119" s="12">
         <v>4999</v>
       </c>
-      <c r="E119" s="17">
+      <c r="E119" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F119" s="17">
+      <c r="F119" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G119" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H119" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I119" s="15">
+      <c r="G119" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H119" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I119" s="14">
         <v>177.0984455958549</v>
       </c>
-      <c r="J119" s="11">
+      <c r="J119" s="10">
         <v>178.47</v>
       </c>
       <c r="K119" s="10">
@@ -4765,34 +4762,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
-      <c r="A120" s="12" t="s">
+      <c r="A120" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B120" s="12" t="s">
+      <c r="B120" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C120" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D120" s="13">
+      <c r="C120" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D120" s="12">
         <v>4999</v>
       </c>
-      <c r="E120" s="17">
+      <c r="E120" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F120" s="17">
+      <c r="F120" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G120" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H120" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I120" s="15">
+      <c r="G120" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H120" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I120" s="14">
         <v>176.946053032612</v>
       </c>
-      <c r="J120" s="11">
+      <c r="J120" s="10">
         <v>178.47</v>
       </c>
       <c r="K120" s="10">
@@ -4800,34 +4797,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
-      <c r="A121" s="12" t="s">
+      <c r="A121" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B121" s="12" t="s">
+      <c r="B121" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C121" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D121" s="13">
+      <c r="C121" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D121" s="12">
         <v>4999</v>
       </c>
-      <c r="E121" s="17">
+      <c r="E121" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F121" s="17">
+      <c r="F121" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G121" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H121" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I121" s="15">
+      <c r="G121" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H121" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I121" s="14">
         <v>176.7936604693691</v>
       </c>
-      <c r="J121" s="11">
+      <c r="J121" s="10">
         <v>178.47</v>
       </c>
       <c r="K121" s="10">
@@ -4847,10 +4844,10 @@
       <c r="D122" s="8">
         <v>4999</v>
       </c>
-      <c r="E122" s="16">
+      <c r="E122" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F122" s="16">
+      <c r="F122" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G122" s="2" t="s">
@@ -4862,7 +4859,7 @@
       <c r="I122" s="10">
         <v>177.5556232855836</v>
       </c>
-      <c r="J122" s="11">
+      <c r="J122" s="10">
         <v>178.47</v>
       </c>
       <c r="K122" s="10">
@@ -4882,10 +4879,10 @@
       <c r="D123" s="8">
         <v>4999</v>
       </c>
-      <c r="E123" s="16">
+      <c r="E123" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F123" s="16">
+      <c r="F123" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G123" s="2" t="s">
@@ -4897,7 +4894,7 @@
       <c r="I123" s="10">
         <v>176.946053032612</v>
       </c>
-      <c r="J123" s="11">
+      <c r="J123" s="10">
         <v>178.47</v>
       </c>
       <c r="K123" s="10">
@@ -4917,10 +4914,10 @@
       <c r="D124" s="8">
         <v>4999</v>
       </c>
-      <c r="E124" s="16">
+      <c r="E124" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F124" s="16">
+      <c r="F124" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G124" s="2" t="s">
@@ -4932,7 +4929,7 @@
       <c r="I124" s="10">
         <v>176.7936604693691</v>
       </c>
-      <c r="J124" s="11">
+      <c r="J124" s="10">
         <v>178.47</v>
       </c>
       <c r="K124" s="10">
@@ -4952,10 +4949,10 @@
       <c r="D125" s="8">
         <v>4999</v>
       </c>
-      <c r="E125" s="16">
+      <c r="E125" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F125" s="16">
+      <c r="F125" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G125" s="2" t="s">
@@ -4967,7 +4964,7 @@
       <c r="I125" s="10">
         <v>176.6412679061262</v>
       </c>
-      <c r="J125" s="11">
+      <c r="J125" s="10">
         <v>178.47</v>
       </c>
       <c r="K125" s="10">
@@ -4975,34 +4972,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
-      <c r="A126" s="12" t="s">
+      <c r="A126" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B126" s="12" t="s">
+      <c r="B126" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C126" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D126" s="13">
+      <c r="C126" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D126" s="12">
         <v>4999</v>
       </c>
-      <c r="E126" s="17">
+      <c r="E126" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F126" s="17">
+      <c r="F126" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G126" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H126" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I126" s="15">
+      <c r="G126" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H126" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I126" s="14">
         <v>177.4032307223407</v>
       </c>
-      <c r="J126" s="11">
+      <c r="J126" s="10">
         <v>178.47</v>
       </c>
       <c r="K126" s="10">
@@ -5010,34 +5007,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
-      <c r="A127" s="12" t="s">
+      <c r="A127" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B127" s="12" t="s">
+      <c r="B127" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C127" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D127" s="13">
+      <c r="C127" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D127" s="12">
         <v>4999</v>
       </c>
-      <c r="E127" s="17">
+      <c r="E127" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F127" s="17">
+      <c r="F127" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G127" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H127" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I127" s="15">
+      <c r="G127" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H127" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I127" s="14">
         <v>176.7936604693691</v>
       </c>
-      <c r="J127" s="11">
+      <c r="J127" s="10">
         <v>178.47</v>
       </c>
       <c r="K127" s="10">
@@ -5045,34 +5042,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
-      <c r="A128" s="12" t="s">
+      <c r="A128" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B128" s="12" t="s">
+      <c r="B128" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C128" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D128" s="13">
+      <c r="C128" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D128" s="12">
         <v>4999</v>
       </c>
-      <c r="E128" s="17">
+      <c r="E128" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F128" s="17">
+      <c r="F128" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G128" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H128" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I128" s="15">
+      <c r="G128" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H128" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I128" s="14">
         <v>176.6412679061262</v>
       </c>
-      <c r="J128" s="11">
+      <c r="J128" s="10">
         <v>178.47</v>
       </c>
       <c r="K128" s="10">
@@ -5080,34 +5077,34 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
-      <c r="A129" s="12" t="s">
+      <c r="A129" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B129" s="12" t="s">
+      <c r="B129" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C129" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D129" s="13">
+      <c r="C129" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D129" s="12">
         <v>4999</v>
       </c>
-      <c r="E129" s="17">
+      <c r="E129" s="16">
         <v>44.6103999999999</v>
       </c>
-      <c r="F129" s="17">
+      <c r="F129" s="16">
         <v>-87.9868</v>
       </c>
-      <c r="G129" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H129" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I129" s="15">
+      <c r="G129" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H129" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I129" s="14">
         <v>176.4888753428832</v>
       </c>
-      <c r="J129" s="11">
+      <c r="J129" s="10">
         <v>178.47</v>
       </c>
       <c r="K129" s="10">
@@ -5127,10 +5124,10 @@
       <c r="D130" s="8">
         <v>4999</v>
       </c>
-      <c r="E130" s="16">
+      <c r="E130" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F130" s="16">
+      <c r="F130" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G130" s="2" t="s">
@@ -5142,7 +5139,7 @@
       <c r="I130" s="10">
         <v>177.2508381590978</v>
       </c>
-      <c r="J130" s="11">
+      <c r="J130" s="10">
         <v>178.47</v>
       </c>
       <c r="K130" s="10">
@@ -5162,10 +5159,10 @@
       <c r="D131" s="8">
         <v>4999</v>
       </c>
-      <c r="E131" s="16">
+      <c r="E131" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F131" s="16">
+      <c r="F131" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G131" s="2" t="s">
@@ -5177,7 +5174,7 @@
       <c r="I131" s="10">
         <v>176.6412679061262</v>
       </c>
-      <c r="J131" s="11">
+      <c r="J131" s="10">
         <v>178.47</v>
       </c>
       <c r="K131" s="10">
@@ -5197,10 +5194,10 @@
       <c r="D132" s="8">
         <v>4999</v>
       </c>
-      <c r="E132" s="16">
+      <c r="E132" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F132" s="16">
+      <c r="F132" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G132" s="2" t="s">
@@ -5212,7 +5209,7 @@
       <c r="I132" s="10">
         <v>176.4888753428832</v>
       </c>
-      <c r="J132" s="11">
+      <c r="J132" s="10">
         <v>178.47</v>
       </c>
       <c r="K132" s="10">
@@ -5232,10 +5229,10 @@
       <c r="D133" s="8">
         <v>4999</v>
       </c>
-      <c r="E133" s="16">
+      <c r="E133" s="15">
         <v>44.6103999999999</v>
       </c>
-      <c r="F133" s="16">
+      <c r="F133" s="15">
         <v>-87.9868</v>
       </c>
       <c r="G133" s="2" t="s">
@@ -5247,7 +5244,7 @@
       <c r="I133" s="10">
         <v>176.3364827796403</v>
       </c>
-      <c r="J133" s="11">
+      <c r="J133" s="10">
         <v>178.47</v>
       </c>
       <c r="K133" s="10">

</xml_diff>